<commit_message>
Cahier de recette : mise a jour apres les retours (21 cas)
- CR-15 a CR-17 : fenetre Voir detail — colonnes Debut/Fin de journee
  (stock rayon ET stock reserve), groupe Interne reserve par jour, jour
  'reserve seule' present, report du stock reserve sur les jours sans
  mouvement (continuite chronologique).
- CR-18 : impression PDF A4 paysage (bouton imprimer).
- CR-02/CR-11 : filtre fabricant retire de l'ecran.
- Prerequis : migrations V6.5.26, V6.5.27 et V6.5.28, cache navigateur.
- CR-21 : performance avec les deux index.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUPb6xU2anUAUr8b3nRbac
</commit_message>
<xml_diff>
--- a/docs/cahier_recette_suivi_mvt_article_complet.xlsx
+++ b/docs/cahier_recette_suivi_mvt_article_complet.xlsx
@@ -20,12 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="116">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="129">
   <si>
     <t xml:space="preserve">CAHIER DE RECETTE — Suivi mouvement article complet (intégration des mouvements de réserve)</t>
   </si>
   <si>
-    <t xml:space="preserve">Application Prestige — branche claude/suivi-mouvement-article-oh1r8i — Prérequis généraux : migrations V6.5.26 (index) et V6.5.27 (menu) exécutées, reconnexion faite, un produit de test suivi en réserve (bool_RESERVE=1) avec stock rayon &gt; 0. L'écran « Suivi mouvement article 2 » reste inchangé.</t>
+    <t xml:space="preserve">Application Prestige — branche claude/suivi-mouvement-article-oh1r8i — Prérequis généraux : migrations V6.5.26 (index réserve), V6.5.27 (menu) et V6.5.28 (index HMvtProduit) exécutées, reconnexion faite, cache navigateur vidé, un produit de test suivi en réserve (bool_RESERVE=1) avec stock rayon &gt; 0. L'écran « Suivi mouvement article 2 » reste inchangé.</t>
   </si>
   <si>
     <t xml:space="preserve">Testeur :</t>
@@ -103,13 +103,13 @@
     <t xml:space="preserve">Écran</t>
   </si>
   <si>
-    <t xml:space="preserve">Toutes les colonnes attendues sont visibles</t>
+    <t xml:space="preserve">Toutes les colonnes attendues sont visibles, sans filtre fabricant</t>
   </si>
   <si>
     <t xml:space="preserve">Ouvrir l'écran, lancer une recherche sur la période du jour.</t>
   </si>
   <si>
-    <t xml:space="preserve">Groupes « Mouvements Sortie », « Mouvements Entrée », « Mouvements internes réserve » (Vers réserve, Vers rayon, Ajust.réserve), colonnes Qté.Inv, écart.Inv, Stock rayon, Stock réserve, Stock total.</t>
+    <t xml:space="preserve">Groupes « Mouvements Sortie », « Mouvements Entrée », « Mouvements internes réserve » (Vers réserve, Vers rayon, Ajust.réserve), colonnes Qté.Inv, écart.Inv, Stock rayon, Stock réserve, Stock total ; le filtre fabricant est absent (retiré de cet écran).</t>
   </si>
   <si>
     <t xml:space="preserve">CR-03</t>
@@ -235,7 +235,7 @@
     <t xml:space="preserve">Tous les filtres s'appliquent aussi aux mouvements internes</t>
   </si>
   <si>
-    <t xml:space="preserve">Tester séparément : période, recherche CIP/nom, famille article, zone géographique, fabricant.</t>
+    <t xml:space="preserve">Tester séparément : période, recherche CIP/nom, famille article, zone géographique.</t>
   </si>
   <si>
     <t xml:space="preserve">Chaque filtre restreint la liste ET les totaux internes ; aucun mouvement hors filtre n'est compté.</t>
@@ -292,18 +292,57 @@
     <t xml:space="preserve">Détail par jour</t>
   </si>
   <si>
-    <t xml:space="preserve">« Voir détail » ouvre le bon produit</t>
+    <t xml:space="preserve">« Voir détail » ouvre le bon produit avec les colonnes complètes</t>
   </si>
   <si>
     <t xml:space="preserve">Faire défiler la grille puis cliquer l'icône détail d'une ligne du bas.</t>
   </si>
   <si>
-    <t xml:space="preserve">Le détail par jour du BON produit s'ouvre (bug du suivi 2 corrigé dans cet écran).</t>
+    <t xml:space="preserve">Le détail du BON produit s'ouvre (bug du suivi 2 corrigé). Colonnes : « Début de journée » (Stock rayon, Stock réserve), Sortie, Entrée, « Interne réserve » (Vers réserve, Vers rayon, Ajust.rés.), Qté.Inv, Ecart.Inv, « Fin de journée » (Stock rayon, Stock réserve) ; totaux Vers réserve / Vers rayon / Ajust.réserve dans le bandeau du bas.</t>
   </si>
   <si>
     <t xml:space="preserve">CR-16</t>
   </si>
   <si>
+    <t xml:space="preserve">Un jour où seule la réserve a bougé apparaît dans le détail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Choisir un jour sans vente/entrée pour le produit ; faire un assort ce jour-là ; ouvrir « Voir détail » sur une période couvrant ce jour.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">La ligne du jour existe : Vers réserve renseigné, colonnes Sortie/Entrée à zéro, stocks rayon début/fin lus dans la trace de réserve (avant du 1er mouvement / après du dernier).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CR-17</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le stock réserve est reporté sur les jours sans mouvement de réserve</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Période de plusieurs jours dont certains sans aucun mouvement de réserve ; comparer les colonnes Stock réserve d'un jour à l'autre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Les jours sans mouvement de réserve affichent le stock réserve du dernier mouvement connu (valeur constante début = fin) ; la chronologie est continue : réserve fin d'un jour = réserve début du suivant.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CR-18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impression</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Le bouton « imprimer » produit un PDF A4 paysage</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filtrer, cliquer « imprimer », examiner le PDF ouvert dans le navigateur, l'imprimer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PDF A4 paysage lisible : en-têtes groupés sur 2 lignes (Sortie / Entrée / Mouvements internes réserve) répétés à chaque page, toutes les lignes filtrées, colonnes Stock rayon / réserve / total.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CR-19</t>
+  </si>
+  <si>
     <t xml:space="preserve">Export</t>
   </si>
   <si>
@@ -316,7 +355,7 @@
     <t xml:space="preserve">Fichier .xls lisible : 20 colonnes dont Vers réserve, Vers rayon, Ajust. réserve et les 3 stocks ; toutes les lignes filtrées, pas seulement la page affichée.</t>
   </si>
   <si>
-    <t xml:space="preserve">CR-17</t>
+    <t xml:space="preserve">CR-20</t>
   </si>
   <si>
     <t xml:space="preserve">Sécurité</t>
@@ -331,19 +370,19 @@
     <t xml:space="preserve">Les deux appels renvoient le message de déconnexion, aucune donnée métier n'est exposée.</t>
   </si>
   <si>
-    <t xml:space="preserve">CR-18</t>
+    <t xml:space="preserve">CR-21</t>
   </si>
   <si>
     <t xml:space="preserve">Performance</t>
   </si>
   <si>
-    <t xml:space="preserve">L'écran reste fluide sur une longue période</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Rechercher 3 mois sans filtre produit sur un volume représentatif (index V6.5.26 posé).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Affichage de la page en moins de 5 secondes ; navigation de pages fluide.</t>
+    <t xml:space="preserve">L'écran et le détail restent fluides sur une longue période</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rechercher 3 mois sans filtre produit sur un volume représentatif (index V6.5.26 et V6.5.28 posés) ; ouvrir un « Voir détail ».</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Affichage de la page en moins de 5 secondes ; navigation de pages et fenêtre de détail fluides.</t>
   </si>
   <si>
     <t xml:space="preserve">SYNTHÈSE (calcul automatique d'après la colonne Statut)</t>
@@ -873,7 +912,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
@@ -989,7 +1028,7 @@
       <c r="F7" s="12"/>
       <c r="G7" s="13"/>
     </row>
-    <row r="8" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
         <v>25</v>
       </c>
@@ -1236,7 +1275,7 @@
       <c r="F20" s="12"/>
       <c r="G20" s="13"/>
     </row>
-    <row r="21" customFormat="false" ht="12" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="49.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="9" t="s">
         <v>88</v>
       </c>
@@ -1255,126 +1294,183 @@
       <c r="F21" s="12"/>
       <c r="G21" s="13"/>
     </row>
-    <row r="22" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="s">
         <v>93</v>
       </c>
       <c r="B22" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>94</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="D22" s="11" t="s">
         <v>95</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="E22" s="11" t="s">
         <v>96</v>
-      </c>
-      <c r="E22" s="11" t="s">
-        <v>97</v>
       </c>
       <c r="F22" s="12"/>
       <c r="G22" s="13"/>
     </row>
-    <row r="23" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="C23" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="D23" s="11" t="s">
         <v>99</v>
       </c>
-      <c r="C23" s="11" t="s">
+      <c r="E23" s="11" t="s">
         <v>100</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>101</v>
-      </c>
-      <c r="E23" s="11" t="s">
-        <v>102</v>
       </c>
       <c r="F23" s="12"/>
       <c r="G23" s="13"/>
     </row>
-    <row r="24" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="B24" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="C24" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="D24" s="11" t="s">
         <v>104</v>
       </c>
-      <c r="C24" s="11" t="s">
+      <c r="E24" s="11" t="s">
         <v>105</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>106</v>
-      </c>
-      <c r="E24" s="11" t="s">
-        <v>107</v>
       </c>
       <c r="F24" s="12"/>
       <c r="G24" s="13"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
+    <row r="25" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>107</v>
+      </c>
+      <c r="C25" s="11" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="14" t="s">
+      <c r="D25" s="11" t="s">
         <v>109</v>
       </c>
-      <c r="B26" s="14" t="s">
+      <c r="E25" s="11" t="s">
         <v>110</v>
       </c>
-      <c r="C26" s="14" t="s">
+      <c r="F25" s="12"/>
+      <c r="G25" s="13"/>
+    </row>
+    <row r="26" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="D26" s="14" t="s">
+      <c r="B26" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="E26" s="14" t="s">
+      <c r="C26" s="11" t="s">
         <v>113</v>
       </c>
-      <c r="F26" s="14" t="s">
+      <c r="D26" s="11" t="s">
         <v>114</v>
       </c>
-      <c r="G26" s="15" t="s">
+      <c r="E26" s="11" t="s">
         <v>115</v>
       </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="16" t="n">
-        <f aca="false">COUNTA(A7:A24)</f>
-        <v>18</v>
-      </c>
-      <c r="B27" s="16" t="n">
-        <f aca="false">COUNTIF(F7:F24,"OK")</f>
+      <c r="F26" s="12"/>
+      <c r="G26" s="13"/>
+    </row>
+    <row r="27" customFormat="false" ht="21" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="9" t="s">
+        <v>116</v>
+      </c>
+      <c r="B27" s="10" t="s">
+        <v>117</v>
+      </c>
+      <c r="C27" s="11" t="s">
+        <v>118</v>
+      </c>
+      <c r="D27" s="11" t="s">
+        <v>119</v>
+      </c>
+      <c r="E27" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="F27" s="12"/>
+      <c r="G27" s="13"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="14" t="s">
+        <v>122</v>
+      </c>
+      <c r="B29" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="D29" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="E29" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="F29" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="G29" s="15" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="16" t="n">
+        <f aca="false">COUNTA(A7:A27)</f>
+        <v>21</v>
+      </c>
+      <c r="B30" s="16" t="n">
+        <f aca="false">COUNTIF(F7:F27,"OK")</f>
         <v>0</v>
       </c>
-      <c r="C27" s="16" t="n">
-        <f aca="false">COUNTIF(F7:F24,"KO")</f>
+      <c r="C30" s="16" t="n">
+        <f aca="false">COUNTIF(F7:F27,"KO")</f>
         <v>0</v>
       </c>
-      <c r="D27" s="16" t="n">
-        <f aca="false">COUNTIF(F7:F24,"NA")</f>
+      <c r="D30" s="16" t="n">
+        <f aca="false">COUNTIF(F7:F27,"NA")</f>
         <v>0</v>
       </c>
-      <c r="E27" s="16" t="n">
-        <f aca="false">A27-B27-C27-D27</f>
-        <v>18</v>
-      </c>
-      <c r="F27" s="17" t="n">
-        <f aca="false">IF(A27=0,0,(B27+C27+D27)/A27)</f>
+      <c r="E30" s="16" t="n">
+        <f aca="false">A30-B30-C30-D30</f>
+        <v>21</v>
+      </c>
+      <c r="F30" s="17" t="n">
+        <f aca="false">IF(A30=0,0,(B30+C30+D30)/A30)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="15"/>
+      <c r="G30" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="3">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
-    <mergeCell ref="G26:G27"/>
+    <mergeCell ref="G29:G30"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Valeurs autorisées : OK, KO ou NA" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F7:F24" type="list">
+    <dataValidation allowBlank="true" error="Valeurs autorisées : OK, KO ou NA" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F7:F27" type="list">
       <formula1>"OK,KO,NA"</formula1>
       <formula2>0</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Renumerotation Flyway apres rebase sur dev : V6.5.26-28 -> V6.7.1-3
dev est desormais a V6.7.0 : nos migrations restaient numeriquement dans
le passe (jouables seulement grace a outOfOrder). Renumerotees a la suite :
V6.7.1 index t_mouvement_reserve, V6.7.2 menu suivi complet, V6.7.3 index
HMvtProduit. Cahier de recette regenere avec les nouveaux numeros
(prerequis et CR-01/CR-21).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BUPb6xU2anUAUr8b3nRbac
</commit_message>
<xml_diff>
--- a/docs/cahier_recette_suivi_mvt_article_complet.xlsx
+++ b/docs/cahier_recette_suivi_mvt_article_complet.xlsx
@@ -25,7 +25,7 @@
     <t xml:space="preserve">CAHIER DE RECETTE — Suivi mouvement article complet (intégration des mouvements de réserve)</t>
   </si>
   <si>
-    <t xml:space="preserve">Application Prestige — branche claude/suivi-mouvement-article-oh1r8i — Prérequis généraux : migrations V6.5.26 (index réserve), V6.5.27 (menu) et V6.5.28 (index HMvtProduit) exécutées, reconnexion faite, cache navigateur vidé, un produit de test suivi en réserve (bool_RESERVE=1) avec stock rayon &gt; 0. L'écran « Suivi mouvement article 2 » reste inchangé.</t>
+    <t xml:space="preserve">Application Prestige — branche claude/suivi-mouvement-article-oh1r8i — Prérequis généraux : migrations V6.7.1 (index réserve), V6.7.2 (menu) et V6.7.3 (index HMvtProduit) exécutées, reconnexion faite, cache navigateur vidé, un produit de test suivi en réserve (bool_RESERVE=1) avec stock rayon &gt; 0. L'écran « Suivi mouvement article 2 » reste inchangé.</t>
   </si>
   <si>
     <t xml:space="preserve">Testeur :</t>
@@ -91,7 +91,7 @@
     <t xml:space="preserve">Le nouveau menu apparaît pour les mêmes profils que le suivi 2</t>
   </si>
   <si>
-    <t xml:space="preserve">Exécuter V6.5.26 et V6.5.27, se reconnecter avec un profil ayant accès au « Suivi mouvement article 2 ».</t>
+    <t xml:space="preserve">Exécuter V6.7.1, V6.7.2 et V6.7.3, se reconnecter avec un profil ayant accès au « Suivi mouvement article 2 ».</t>
   </si>
   <si>
     <t xml:space="preserve">L'entrée « Suivi mouvement article complet » apparaît sous le même menu parent ; l'écran s'ouvre sans erreur.</t>
@@ -379,7 +379,7 @@
     <t xml:space="preserve">L'écran et le détail restent fluides sur une longue période</t>
   </si>
   <si>
-    <t xml:space="preserve">Rechercher 3 mois sans filtre produit sur un volume représentatif (index V6.5.26 et V6.5.28 posés) ; ouvrir un « Voir détail ».</t>
+    <t xml:space="preserve">Rechercher 3 mois sans filtre produit sur un volume représentatif (index V6.7.1 et V6.7.3 posés) ; ouvrir un « Voir détail ».</t>
   </si>
   <si>
     <t xml:space="preserve">Affichage de la page en moins de 5 secondes ; navigation de pages et fenêtre de détail fluides.</t>

</xml_diff>